<commit_message>
update dataset and add report file
</commit_message>
<xml_diff>
--- a/dataset.xlsx
+++ b/dataset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\intern\Sarochinee\งาน\PJ Intern\Code-PJ\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell\Desktop\Code-PJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37E13044-0464-4E59-80F9-5B500F876418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FFB238-26F5-49A0-A8D5-512350B55973}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="1185" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,6 @@
     <t>Model</t>
   </si>
   <si>
-    <t>192.168.0.55</t>
-  </si>
-  <si>
     <t>Username</t>
   </si>
   <si>
@@ -74,6 +71,9 @@
   </si>
   <si>
     <t>H3C</t>
+  </si>
+  <si>
+    <t>192.168.100.120</t>
   </si>
 </sst>
 </file>
@@ -466,10 +466,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
@@ -477,64 +477,64 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
         <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
         <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
         <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="E9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>